<commit_message>
fix optics last deploy version final
</commit_message>
<xml_diff>
--- a/حركات_الشركات_منظمة/البصريات/حركات_ARCAD.xlsx
+++ b/حركات_الشركات_منظمة/البصريات/حركات_ARCAD.xlsx
@@ -1,17 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{301B4143-E51F-4E2A-B20E-6EE34A02C5EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="النظارات" state="visible" r:id="rId4"/>
+    <sheet name="النظارات" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="61">
   <si>
     <t>اسم المريض</t>
   </si>
@@ -109,7 +113,7 @@
     <t>ARCAD006</t>
   </si>
   <si>
-    <t xml:space="preserve"> 12/4/2026</t>
+    <t> 12/4/2026</t>
   </si>
   <si>
     <t xml:space="preserve"> مني رجب محمد </t>
@@ -121,7 +125,7 @@
     <t>ARCAD007</t>
   </si>
   <si>
-    <t xml:space="preserve"> 18/4/2026</t>
+    <t> 18/4/2026</t>
   </si>
   <si>
     <t xml:space="preserve">محمد السيد سليمان </t>
@@ -194,38 +198,31 @@
   </si>
   <si>
     <t>ARCAD014</t>
-  </si>
-  <si>
-    <t>ARCAD2025</t>
-  </si>
-  <si>
-    <t>ARCAD00</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="2">
@@ -596,9 +593,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F44"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.69921875" customWidth="1"/>
     <col min="2" max="2" width="35.09765625" customWidth="1"/>
@@ -910,345 +907,8 @@
         <v>24</v>
       </c>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B16" t="s">
-        <v>61</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B17" t="s">
-        <v>61</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B18" t="s">
-        <v>61</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B19" t="s">
-        <v>61</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B20" t="s">
-        <v>61</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B21" t="s">
-        <v>61</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B22" t="s">
-        <v>61</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B24" t="s">
-        <v>61</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B25" t="s">
-        <v>61</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B26" t="s">
-        <v>61</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B27" t="s">
-        <v>61</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B28" t="s">
-        <v>61</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="29" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B29" t="s">
-        <v>61</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="30" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B30" t="s">
-        <v>61</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="31" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B31" t="s">
-        <v>61</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="32" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B32" t="s">
-        <v>61</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B33" t="s">
-        <v>61</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B34" t="s">
-        <v>61</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B35" t="s">
-        <v>61</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B36" t="s">
-        <v>61</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D36" t="s">
-        <v>63</v>
-      </c>
-      <c r="E36" t="s">
-        <v>63</v>
-      </c>
-      <c r="F36" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>63</v>
-      </c>
-      <c r="B37" t="s">
-        <v>61</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D37" t="s">
-        <v>63</v>
-      </c>
-      <c r="E37" t="s">
-        <v>63</v>
-      </c>
-      <c r="F37" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>63</v>
-      </c>
-      <c r="B38" t="s">
-        <v>61</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D38" t="s">
-        <v>63</v>
-      </c>
-      <c r="E38" t="s">
-        <v>63</v>
-      </c>
-      <c r="F38" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>63</v>
-      </c>
-      <c r="B39" t="s">
-        <v>61</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D39" t="s">
-        <v>63</v>
-      </c>
-      <c r="E39" t="s">
-        <v>63</v>
-      </c>
-      <c r="F39" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>63</v>
-      </c>
-      <c r="B40" t="s">
-        <v>61</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D40" t="s">
-        <v>63</v>
-      </c>
-      <c r="E40" t="s">
-        <v>63</v>
-      </c>
-      <c r="F40" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>63</v>
-      </c>
-      <c r="B41" t="s">
-        <v>61</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D41" t="s">
-        <v>63</v>
-      </c>
-      <c r="E41" t="s">
-        <v>63</v>
-      </c>
-      <c r="F41" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>63</v>
-      </c>
-      <c r="B42" t="s">
-        <v>61</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D42" t="s">
-        <v>63</v>
-      </c>
-      <c r="E42" t="s">
-        <v>63</v>
-      </c>
-      <c r="F42" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>63</v>
-      </c>
-      <c r="B43" t="s">
-        <v>61</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D43" t="s">
-        <v>63</v>
-      </c>
-      <c r="E43" t="s">
-        <v>63</v>
-      </c>
-      <c r="F43" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>63</v>
-      </c>
-      <c r="B44" t="s">
-        <v>61</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="D44" t="s">
-        <v>63</v>
-      </c>
-      <c r="E44" t="s">
-        <v>63</v>
-      </c>
-      <c r="F44" t="s">
-        <v>63</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>